<commit_message>
Project Example 1 - Bank Rating is saved.
</commit_message>
<xml_diff>
--- a/DESIGN/rules/Example 1 - Bank Rating/Bank Rating.xlsx
+++ b/DESIGN/rules/Example 1 - Bank Rating/Bank Rating.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ekosolapova/.openl/user-workspace/ekosolapova/Example 1 - Bank Rating/"/>
     </mc:Choice>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="675">
   <si>
     <t>www.commerzbank.com</t>
   </si>
@@ -6118,10 +6118,10 @@
     </border>
   </borders>
   <cellStyleXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="3"/>
   </cellStyleXfs>
   <cellXfs count="210">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -7154,19 +7154,19 @@
   <sheetPr>
     <tabColor rgb="FF558ED5"/>
   </sheetPr>
-  <dimension ref="A1:AMJ96"/>
+  <dimension ref="B1:J96"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="9.19921875" style="1"/>
-    <col min="3" max="3" width="8.59765625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.59765625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="25.59765625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="42.3984375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="76.59765625" style="1" customWidth="1"/>
-    <col min="8" max="9" width="5.796875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="25" style="1" customWidth="1"/>
-    <col min="11" max="11" width="19.19921875" style="1" customWidth="1"/>
-    <col min="12" max="1024" width="9.19921875" style="1"/>
+    <col min="1" max="2" style="1" width="9.19921875"/>
+    <col min="3" max="3" customWidth="true" style="1" width="8.59765625"/>
+    <col min="4" max="4" customWidth="true" style="1" width="16.59765625"/>
+    <col min="5" max="5" customWidth="true" style="1" width="25.59765625"/>
+    <col min="6" max="6" customWidth="true" style="1" width="42.3984375"/>
+    <col min="7" max="7" customWidth="true" style="1" width="76.59765625"/>
+    <col min="8" max="9" customWidth="true" style="1" width="5.796875"/>
+    <col min="10" max="10" customWidth="true" style="1" width="25.0"/>
+    <col min="11" max="11" customWidth="true" style="1" width="19.19921875"/>
+    <col min="12" max="1024" style="1" width="9.19921875"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="15" x14ac:dyDescent="0.2">
@@ -8166,9 +8166,9 @@
   <dimension ref="B3:E25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="27.19921875" customWidth="1"/>
-    <col min="4" max="4" width="27.3984375" customWidth="1"/>
-    <col min="5" max="5" width="31.59765625" customWidth="1"/>
+    <col min="3" max="3" customWidth="true" width="27.19921875"/>
+    <col min="4" max="4" customWidth="true" width="27.3984375"/>
+    <col min="5" max="5" customWidth="true" width="31.59765625"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:5" ht="20" x14ac:dyDescent="0.25">
@@ -8349,9 +8349,9 @@
   <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="31.59765625" customWidth="1"/>
-    <col min="5" max="5" width="36" customWidth="1"/>
+    <col min="3" max="3" customWidth="true" width="25.0"/>
+    <col min="4" max="4" customWidth="true" width="31.59765625"/>
+    <col min="5" max="5" customWidth="true" width="36.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -8478,8 +8478,8 @@
   <dimension ref="C3:D13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="22.59765625" customWidth="1"/>
-    <col min="4" max="4" width="25.59765625" customWidth="1"/>
+    <col min="3" max="3" customWidth="true" width="22.59765625"/>
+    <col min="4" max="4" customWidth="true" width="25.59765625"/>
   </cols>
   <sheetData>
     <row r="3" spans="3:4" ht="20" x14ac:dyDescent="0.25">
@@ -8566,15 +8566,15 @@
   <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.3984375" customWidth="1"/>
-    <col min="2" max="2" width="3.796875" customWidth="1"/>
-    <col min="3" max="3" width="9.796875" customWidth="1"/>
-    <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="5" width="30.796875" customWidth="1"/>
-    <col min="6" max="6" width="11.59765625" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="11.59765625" customWidth="1"/>
-    <col min="9" max="9" width="11" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="4.3984375"/>
+    <col min="2" max="2" customWidth="true" width="3.796875"/>
+    <col min="3" max="3" customWidth="true" width="9.796875"/>
+    <col min="4" max="4" customWidth="true" width="24.0"/>
+    <col min="5" max="5" customWidth="true" width="30.796875"/>
+    <col min="6" max="6" customWidth="true" width="11.59765625"/>
+    <col min="7" max="7" customWidth="true" width="12.0"/>
+    <col min="8" max="8" customWidth="true" width="11.59765625"/>
+    <col min="9" max="9" customWidth="true" width="11.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
@@ -8664,178 +8664,104 @@
       <c r="I12" s="80"/>
     </row>
     <row r="13" spans="1:9" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="110">
-        <v>1</v>
-      </c>
-      <c r="D13" s="172"/>
-      <c r="E13" s="174"/>
-      <c r="F13" s="174"/>
-      <c r="G13" s="174"/>
-      <c r="H13" s="174"/>
-      <c r="I13" s="174"/>
+      <c r="C13" t="n" s="111">
+        <v>7.0</v>
+      </c>
+      <c r="D13" t="s" s="74">
+        <v>667</v>
+      </c>
+      <c r="E13" t="n" s="83">
+        <v>1.0</v>
+      </c>
+      <c r="F13" t="n" s="83">
+        <v>0.25</v>
+      </c>
+      <c r="G13" t="n" s="83">
+        <v>0.8</v>
+      </c>
+      <c r="H13" t="n" s="83">
+        <v>1.0</v>
+      </c>
+      <c r="I13" t="n" s="51">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="111">
-        <v>2</v>
-      </c>
-      <c r="D14" s="172"/>
-      <c r="E14" s="175"/>
-      <c r="F14" s="173"/>
-      <c r="G14" s="173"/>
-      <c r="H14" s="173"/>
-      <c r="I14" s="173"/>
+      <c r="C14" s="111" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="D14" s="74" t="s">
+        <v>666</v>
+      </c>
+      <c r="E14" s="83" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F14" s="83" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G14" s="83" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H14" s="83" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="I14" s="51" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C15" s="111">
-        <v>3</v>
-      </c>
-      <c r="D15" s="176"/>
-      <c r="E15" s="175"/>
-      <c r="F15" s="173"/>
-      <c r="G15" s="173"/>
-      <c r="H15" s="173"/>
-      <c r="I15" s="173"/>
+      <c r="C15" s="111" t="n">
+        <v>9.0</v>
+      </c>
+      <c r="D15" s="74" t="s">
+        <v>665</v>
+      </c>
+      <c r="E15" s="83" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F15" s="83" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="G15" s="83" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H15" s="83" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I15" s="51" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C16" s="111">
-        <v>4</v>
-      </c>
-      <c r="D16" s="177" t="s">
-        <v>668</v>
-      </c>
-      <c r="E16" s="175"/>
-      <c r="F16" s="173"/>
-      <c r="G16" s="173"/>
-      <c r="H16" s="173"/>
-      <c r="I16" s="173"/>
-    </row>
-    <row r="17" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C17" s="111">
-        <v>5</v>
-      </c>
-      <c r="D17" s="177"/>
-      <c r="E17" s="175"/>
-      <c r="F17" s="173"/>
-      <c r="G17" s="173"/>
-      <c r="H17" s="173"/>
-      <c r="I17" s="173"/>
-    </row>
-    <row r="18" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C18" s="111">
-        <v>6</v>
-      </c>
-      <c r="D18" s="178"/>
-      <c r="E18" s="175"/>
-      <c r="F18" s="173"/>
-      <c r="G18" s="173"/>
-      <c r="H18" s="173"/>
-      <c r="I18" s="173"/>
-    </row>
-    <row r="19" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C19" s="111">
-        <v>7</v>
-      </c>
-      <c r="D19" s="74" t="s">
-        <v>667</v>
-      </c>
-      <c r="E19" s="83">
-        <v>1</v>
-      </c>
-      <c r="F19" s="83">
+      <c r="C16" s="111" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="D16" s="109" t="s">
+        <v>664</v>
+      </c>
+      <c r="E16" s="83" t="n">
         <v>0.25</v>
       </c>
-      <c r="G19" s="83">
-        <v>0.8</v>
-      </c>
-      <c r="H19" s="83">
-        <v>1</v>
-      </c>
-      <c r="I19" s="51">
+      <c r="F16" s="83" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G16" s="83" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H16" s="83" t="n">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="20" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C20" s="111">
-        <v>8</v>
-      </c>
-      <c r="D20" s="74" t="s">
-        <v>666</v>
-      </c>
-      <c r="E20" s="83">
-        <v>0.9</v>
-      </c>
-      <c r="F20" s="83">
-        <v>0.15</v>
-      </c>
-      <c r="G20" s="83">
-        <v>0.7</v>
-      </c>
-      <c r="H20" s="83">
-        <v>1</v>
-      </c>
-      <c r="I20" s="51">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="21" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C21" s="111">
-        <v>9</v>
-      </c>
-      <c r="D21" s="74" t="s">
-        <v>665</v>
-      </c>
-      <c r="E21" s="83">
-        <v>0.7</v>
-      </c>
-      <c r="F21" s="83">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="G21" s="83">
-        <v>0.5</v>
-      </c>
-      <c r="H21" s="83">
-        <v>0.9</v>
-      </c>
-      <c r="I21" s="51">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="22" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C22" s="111">
-        <v>10</v>
-      </c>
-      <c r="D22" s="109" t="s">
-        <v>664</v>
-      </c>
-      <c r="E22" s="83">
-        <v>0.25</v>
-      </c>
-      <c r="F22" s="83">
-        <v>0.01</v>
-      </c>
-      <c r="G22" s="83">
-        <v>0.25</v>
-      </c>
-      <c r="H22" s="83">
-        <v>0.7</v>
-      </c>
-      <c r="I22" s="51">
+      <c r="I16" s="51" t="n">
         <v>0.02</v>
       </c>
     </row>
-    <row r="23" spans="3:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="112">
-        <v>11</v>
-      </c>
-      <c r="D23" s="67" t="s">
-        <v>663</v>
-      </c>
-      <c r="E23" s="179"/>
-      <c r="F23" s="179"/>
-      <c r="G23" s="179"/>
-      <c r="H23" s="179"/>
-      <c r="I23" s="179"/>
-    </row>
+    <row r="17" spans="3:9" x14ac:dyDescent="0.2"/>
+    <row r="18" spans="3:9" x14ac:dyDescent="0.2"/>
+    <row r="19" spans="3:9" x14ac:dyDescent="0.2"/>
+    <row r="20" spans="3:9" x14ac:dyDescent="0.2"/>
+    <row r="21" spans="3:9" x14ac:dyDescent="0.2"/>
+    <row r="22" spans="3:9" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="3:9" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="3:9" x14ac:dyDescent="0.2">
       <c r="D28" s="169"/>
     </row>
@@ -8875,9 +8801,9 @@
   <dimension ref="C3:E9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="20.59765625" customWidth="1"/>
-    <col min="4" max="4" width="30.59765625" customWidth="1"/>
-    <col min="5" max="5" width="19.3984375" customWidth="1"/>
+    <col min="3" max="3" customWidth="true" width="20.59765625"/>
+    <col min="4" max="4" customWidth="true" width="30.59765625"/>
+    <col min="5" max="5" customWidth="true" width="19.3984375"/>
   </cols>
   <sheetData>
     <row r="3" spans="3:5" ht="20" x14ac:dyDescent="0.25">
@@ -8946,14 +8872,14 @@
   <sheetPr>
     <tabColor rgb="FF8EB4E3"/>
   </sheetPr>
-  <dimension ref="A1:AMJ8"/>
+  <dimension ref="B1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="9.19921875" style="72"/>
-    <col min="3" max="3" width="18.19921875" style="72" customWidth="1"/>
-    <col min="4" max="4" width="13.59765625" style="72" customWidth="1"/>
-    <col min="5" max="5" width="14" style="72" customWidth="1"/>
-    <col min="6" max="1024" width="9.19921875" style="72"/>
+    <col min="1" max="2" style="72" width="9.19921875"/>
+    <col min="3" max="3" customWidth="true" style="72" width="18.19921875"/>
+    <col min="4" max="4" customWidth="true" style="72" width="13.59765625"/>
+    <col min="5" max="5" customWidth="true" style="72" width="14.0"/>
+    <col min="6" max="1024" style="72" width="9.19921875"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6" x14ac:dyDescent="0.2">
@@ -9020,8 +8946,8 @@
   <dimension ref="B1:E21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="28.3984375" customWidth="1"/>
-    <col min="4" max="4" width="76.19921875" customWidth="1"/>
+    <col min="3" max="3" customWidth="true" width="28.3984375"/>
+    <col min="4" max="4" customWidth="true" width="76.19921875"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:5" x14ac:dyDescent="0.2">
@@ -9181,8 +9107,8 @@
   <dimension ref="C3:D13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="20.3984375" customWidth="1"/>
-    <col min="4" max="4" width="26.19921875" customWidth="1"/>
+    <col min="3" max="3" customWidth="true" width="20.3984375"/>
+    <col min="4" max="4" customWidth="true" width="26.19921875"/>
   </cols>
   <sheetData>
     <row r="3" spans="3:4" ht="20" x14ac:dyDescent="0.25">
@@ -9246,13 +9172,13 @@
   <sheetPr>
     <tabColor rgb="FFEEECE1"/>
   </sheetPr>
-  <dimension ref="A2:AMJ49"/>
+  <dimension ref="B2:E49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="9.19921875" style="72"/>
-    <col min="3" max="3" width="17.59765625" style="72" customWidth="1"/>
-    <col min="4" max="4" width="39.19921875" style="72" customWidth="1"/>
-    <col min="5" max="1024" width="9.19921875" style="72"/>
+    <col min="1" max="2" style="72" width="9.19921875"/>
+    <col min="3" max="3" customWidth="true" style="72" width="17.59765625"/>
+    <col min="4" max="4" customWidth="true" style="72" width="39.19921875"/>
+    <col min="5" max="1024" style="72" width="9.19921875"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="20" x14ac:dyDescent="0.25">
@@ -9669,13 +9595,13 @@
     <tabColor rgb="FFC6D9F1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A3:AMJ85"/>
+  <dimension ref="B3:D85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="3" width="9.19921875" style="72"/>
-    <col min="4" max="4" width="34.3984375" style="72" customWidth="1"/>
-    <col min="5" max="5" width="30" style="72" customWidth="1"/>
-    <col min="6" max="1024" width="9.19921875" style="72"/>
+    <col min="1" max="3" style="72" width="9.19921875"/>
+    <col min="4" max="4" customWidth="true" style="72" width="34.3984375"/>
+    <col min="5" max="5" customWidth="true" style="72" width="30.0"/>
+    <col min="6" max="1024" style="72" width="9.19921875"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:4" ht="20" x14ac:dyDescent="0.25">
@@ -10066,9 +9992,9 @@
   <dimension ref="A3:E43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="21.3984375" customWidth="1"/>
-    <col min="4" max="4" width="38" customWidth="1"/>
-    <col min="5" max="5" width="22.19921875" customWidth="1"/>
+    <col min="3" max="3" customWidth="true" width="21.3984375"/>
+    <col min="4" max="4" customWidth="true" width="38.0"/>
+    <col min="5" max="5" customWidth="true" width="22.19921875"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:5" ht="20" x14ac:dyDescent="0.25">
@@ -10321,30 +10247,30 @@
   <sheetPr>
     <tabColor rgb="FFC6D9F1"/>
   </sheetPr>
-  <dimension ref="A2:AMJ90"/>
+  <dimension ref="B2:S90"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.59765625" style="72" customWidth="1"/>
-    <col min="2" max="2" width="9.19921875" style="72"/>
-    <col min="3" max="3" width="19.19921875" style="72" customWidth="1"/>
-    <col min="4" max="4" width="21" style="72" customWidth="1"/>
-    <col min="5" max="5" width="28.3984375" style="72" customWidth="1"/>
-    <col min="6" max="6" width="25" style="72" customWidth="1"/>
-    <col min="7" max="7" width="51.59765625" style="72" customWidth="1"/>
-    <col min="8" max="8" width="30.19921875" style="72" customWidth="1"/>
-    <col min="9" max="9" width="32.59765625" style="72" customWidth="1"/>
-    <col min="10" max="10" width="48.59765625" style="72" customWidth="1"/>
-    <col min="11" max="11" width="29.796875" style="72" customWidth="1"/>
-    <col min="12" max="12" width="9.59765625" style="72" customWidth="1"/>
-    <col min="13" max="13" width="10" style="72" customWidth="1"/>
-    <col min="14" max="14" width="12.3984375" style="72" customWidth="1"/>
-    <col min="15" max="15" width="21.59765625" style="72" customWidth="1"/>
-    <col min="16" max="16" width="25.796875" style="72" customWidth="1"/>
-    <col min="17" max="17" width="25" style="72" customWidth="1"/>
-    <col min="18" max="18" width="38.59765625" style="72" customWidth="1"/>
-    <col min="19" max="19" width="23.19921875" style="72" customWidth="1"/>
-    <col min="20" max="20" width="19.3984375" style="72" customWidth="1"/>
-    <col min="21" max="1024" width="9.19921875" style="72"/>
+    <col min="1" max="1" customWidth="true" style="72" width="3.59765625"/>
+    <col min="2" max="2" style="72" width="9.19921875"/>
+    <col min="3" max="3" customWidth="true" style="72" width="19.19921875"/>
+    <col min="4" max="4" customWidth="true" style="72" width="21.0"/>
+    <col min="5" max="5" customWidth="true" style="72" width="28.3984375"/>
+    <col min="6" max="6" customWidth="true" style="72" width="25.0"/>
+    <col min="7" max="7" customWidth="true" style="72" width="51.59765625"/>
+    <col min="8" max="8" customWidth="true" style="72" width="30.19921875"/>
+    <col min="9" max="9" customWidth="true" style="72" width="32.59765625"/>
+    <col min="10" max="10" customWidth="true" style="72" width="48.59765625"/>
+    <col min="11" max="11" customWidth="true" style="72" width="29.796875"/>
+    <col min="12" max="12" customWidth="true" style="72" width="9.59765625"/>
+    <col min="13" max="13" customWidth="true" style="72" width="10.0"/>
+    <col min="14" max="14" customWidth="true" style="72" width="12.3984375"/>
+    <col min="15" max="15" customWidth="true" style="72" width="21.59765625"/>
+    <col min="16" max="16" customWidth="true" style="72" width="25.796875"/>
+    <col min="17" max="17" customWidth="true" style="72" width="25.0"/>
+    <col min="18" max="18" customWidth="true" style="72" width="38.59765625"/>
+    <col min="19" max="19" customWidth="true" style="72" width="23.19921875"/>
+    <col min="20" max="20" customWidth="true" style="72" width="19.3984375"/>
+    <col min="21" max="1024" style="72" width="9.19921875"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:19" ht="20" x14ac:dyDescent="0.25">
@@ -11546,10 +11472,10 @@
   <dimension ref="A1:I116"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.19921875" customWidth="1"/>
-    <col min="3" max="3" width="43.59765625" customWidth="1"/>
-    <col min="4" max="4" width="34.3984375" customWidth="1"/>
-    <col min="5" max="5" width="9.796875" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="9.19921875"/>
+    <col min="3" max="3" customWidth="true" width="43.59765625"/>
+    <col min="4" max="4" customWidth="true" width="34.3984375"/>
+    <col min="5" max="5" customWidth="true" width="9.796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
@@ -12254,10 +12180,10 @@
   <dimension ref="B3:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="14.19921875" customWidth="1"/>
-    <col min="3" max="3" width="23.19921875" customWidth="1"/>
-    <col min="4" max="4" width="27.19921875" customWidth="1"/>
-    <col min="5" max="5" width="24.59765625" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="14.19921875"/>
+    <col min="3" max="3" customWidth="true" width="23.19921875"/>
+    <col min="4" max="4" customWidth="true" width="27.19921875"/>
+    <col min="5" max="5" customWidth="true" width="24.59765625"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:4" ht="20" x14ac:dyDescent="0.25">
@@ -12337,9 +12263,9 @@
   <dimension ref="A3:G42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="31.59765625" customWidth="1"/>
-    <col min="5" max="5" width="26.3984375" customWidth="1"/>
+    <col min="3" max="3" customWidth="true" width="30.0"/>
+    <col min="4" max="4" customWidth="true" width="31.59765625"/>
+    <col min="5" max="5" customWidth="true" width="26.3984375"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:7" ht="20" x14ac:dyDescent="0.25">
@@ -12608,9 +12534,9 @@
   <dimension ref="B3:E12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="14.796875" customWidth="1"/>
-    <col min="4" max="4" width="23.19921875" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="3" max="3" customWidth="true" width="14.796875"/>
+    <col min="4" max="4" customWidth="true" width="23.19921875"/>
+    <col min="5" max="5" customWidth="true" width="22.0"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:5" ht="20" x14ac:dyDescent="0.25">
@@ -12710,8 +12636,8 @@
   <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="4" width="31.3984375" customWidth="1"/>
-    <col min="5" max="5" width="22.19921875" customWidth="1"/>
+    <col min="3" max="4" customWidth="true" width="31.3984375"/>
+    <col min="5" max="5" customWidth="true" width="22.19921875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -13037,9 +12963,9 @@
   <dimension ref="B3:I20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="18.796875" customWidth="1"/>
-    <col min="4" max="4" width="22.3984375" customWidth="1"/>
-    <col min="5" max="5" width="21.59765625" customWidth="1"/>
+    <col min="3" max="3" customWidth="true" width="18.796875"/>
+    <col min="4" max="4" customWidth="true" width="22.3984375"/>
+    <col min="5" max="5" customWidth="true" width="21.59765625"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:9" ht="20" x14ac:dyDescent="0.25">
@@ -13179,12 +13105,12 @@
   <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.19921875" customWidth="1"/>
-    <col min="3" max="3" width="44.796875" customWidth="1"/>
-    <col min="4" max="4" width="40.3984375" customWidth="1"/>
-    <col min="5" max="5" width="35.3984375" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="8" max="8" width="26.3984375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="9.19921875"/>
+    <col min="3" max="3" customWidth="true" width="44.796875"/>
+    <col min="4" max="4" customWidth="true" width="40.3984375"/>
+    <col min="5" max="5" customWidth="true" width="35.3984375"/>
+    <col min="6" max="6" customWidth="true" width="15.0"/>
+    <col min="8" max="8" customWidth="true" width="26.3984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>